<commit_message>
Integrei com o framework flask;
agora as variaveis recebem valor pelo html atraves de funcoes
</commit_message>
<xml_diff>
--- a/Pasta1.xlsx
+++ b/Pasta1.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>aa</t>
+          <t>a</t>
         </is>
       </c>
       <c r="C6" s="2" t="n"/>
@@ -885,7 +885,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>aa</t>
         </is>
       </c>
       <c r="C7" s="2" t="n"/>
@@ -963,7 +963,7 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>aa</t>
         </is>
       </c>
       <c r="C9" s="2" t="n"/>

</xml_diff>